<commit_message>
update 3 pathway 270126
</commit_message>
<xml_diff>
--- a/ssp_modeling/transformations/templates/calibrated/mexico/model_input_variables_mexico_se_calibrated.xlsx
+++ b/ssp_modeling/transformations/templates/calibrated/mexico/model_input_variables_mexico_se_calibrated.xlsx
@@ -10,15 +10,13 @@
     <sheet name="strategy_id-0" sheetId="1" r:id="rId1"/>
     <sheet name="strategy_id-6004" sheetId="2" r:id="rId2"/>
     <sheet name="strategy_id-6005" sheetId="3" r:id="rId3"/>
-    <sheet name="strategy_id-6006" sheetId="4" r:id="rId4"/>
-    <sheet name="strategy_id-6007" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="68">
   <si>
     <t>subsector</t>
   </si>
@@ -787,118 +785,118 @@
         <v>2582.57</v>
       </c>
       <c r="R2">
-        <v>2665.9611853</v>
+        <v>2665.961185</v>
       </c>
       <c r="S2">
-        <v>2729.064486556051</v>
+        <v>2729.064487</v>
       </c>
       <c r="T2">
-        <v>2768.308433872728</v>
+        <v>2768.308434</v>
       </c>
       <c r="U2">
-        <v>2821.875202068165</v>
+        <v>2821.875202</v>
       </c>
       <c r="V2">
-        <v>2879.892956222686</v>
+        <v>2879.892956</v>
       </c>
       <c r="W2">
-        <v>2939.247550050436</v>
+        <v>2939.24755</v>
       </c>
       <c r="X2">
-        <v>2999.825442056975</v>
+        <v>2999.825442</v>
       </c>
       <c r="Y2">
-        <v>3064.774014262171</v>
+        <v>3064.774014</v>
       </c>
       <c r="Z2">
-        <v>3133.687620037442</v>
+        <v>3133.68762</v>
       </c>
       <c r="AA2">
-        <v>3206.767180385722</v>
+        <v>3206.76718</v>
       </c>
       <c r="AB2">
-        <v>3284.228401143724</v>
+        <v>3284.228401</v>
       </c>
       <c r="AC2">
-        <v>3366.302813475037</v>
+        <v>3366.302813</v>
       </c>
       <c r="AD2">
-        <v>3453.238902955263</v>
+        <v>3453.238903</v>
       </c>
       <c r="AE2">
-        <v>3545.303334823448</v>
+        <v>3545.303335</v>
       </c>
       <c r="AF2">
-        <v>3642.782283700117</v>
+        <v>3642.782284</v>
       </c>
       <c r="AG2">
-        <v>3745.982876869395</v>
+        <v>3745.982877</v>
       </c>
       <c r="AH2">
-        <v>3854.879962573155</v>
+        <v>3854.879963</v>
       </c>
       <c r="AI2">
-        <v>3969.092768170632</v>
+        <v>3969.092768</v>
       </c>
       <c r="AJ2">
-        <v>4086.265089172769</v>
+        <v>4086.265089</v>
       </c>
       <c r="AK2">
-        <v>4206.035987881747</v>
+        <v>4206.035988</v>
       </c>
       <c r="AL2">
-        <v>4327.620495817171</v>
+        <v>4327.620496</v>
       </c>
       <c r="AM2">
-        <v>4451.175014664492</v>
+        <v>4451.175015</v>
       </c>
       <c r="AN2">
-        <v>4576.865801935641</v>
+        <v>4576.865802</v>
       </c>
       <c r="AO2">
-        <v>4704.294963972647</v>
+        <v>4704.294964</v>
       </c>
       <c r="AP2">
-        <v>4833.390311373371</v>
+        <v>4833.390311</v>
       </c>
       <c r="AQ2">
-        <v>4964.666776420458</v>
+        <v>4964.666776</v>
       </c>
       <c r="AR2">
-        <v>5098.813058875173</v>
+        <v>5098.813059</v>
       </c>
       <c r="AS2">
-        <v>5236.227042493289</v>
+        <v>5236.227042</v>
       </c>
       <c r="AT2">
-        <v>5376.450595080234</v>
+        <v>5376.450595</v>
       </c>
       <c r="AU2">
-        <v>5519.036629803664</v>
+        <v>5519.03663</v>
       </c>
       <c r="AV2">
-        <v>5662.966874751141</v>
+        <v>5662.966875</v>
       </c>
       <c r="AW2">
-        <v>5808.25799981783</v>
+        <v>5808.258</v>
       </c>
       <c r="AX2">
-        <v>5953.944544307815</v>
+        <v>5953.944544</v>
       </c>
       <c r="AY2">
-        <v>6100.132250634922</v>
+        <v>6100.132251</v>
       </c>
       <c r="AZ2">
-        <v>6247.477018321883</v>
+        <v>6247.477018</v>
       </c>
       <c r="BA2">
-        <v>6396.056995700144</v>
+        <v>6396.056996</v>
       </c>
       <c r="BB2">
-        <v>6546.507371564338</v>
+        <v>6546.507372</v>
       </c>
       <c r="BC2">
-        <v>6699.483598533054</v>
+        <v>6699.483599</v>
       </c>
     </row>
     <row r="3" spans="1:55">
@@ -1979,142 +1977,142 @@
         <v>1</v>
       </c>
       <c r="J10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="K10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="L10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="M10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="N10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="O10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="P10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="Q10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="R10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="S10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="T10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="U10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="V10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="W10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="X10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="Y10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="Z10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AA10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AB10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AC10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AD10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AE10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AF10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AG10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AH10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AI10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AJ10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AK10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AL10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AM10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AN10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AO10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AP10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AQ10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AR10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AS10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AT10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AU10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AV10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AW10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AX10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AY10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="AZ10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="BA10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="BB10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
       <c r="BC10">
-        <v>3.981666666666667</v>
+        <v>3.981666667</v>
       </c>
     </row>
     <row r="11" spans="1:55">
@@ -2131,142 +2129,142 @@
         <v>1</v>
       </c>
       <c r="J11">
-        <v>25242936.69465</v>
+        <v>25242936.69</v>
       </c>
       <c r="K11">
-        <v>25188375.99317</v>
+        <v>25188375.99</v>
       </c>
       <c r="L11">
-        <v>25121419.04358</v>
+        <v>25121419.04</v>
       </c>
       <c r="M11">
-        <v>25041298.78008</v>
+        <v>25041298.78</v>
       </c>
       <c r="N11">
-        <v>24948670.45124</v>
+        <v>24948670.45</v>
       </c>
       <c r="O11">
-        <v>24844052.17557</v>
+        <v>24844052.18</v>
       </c>
       <c r="P11">
-        <v>24148167.4605303</v>
+        <v>24148167.46</v>
       </c>
       <c r="Q11">
-        <v>23982180.0528006</v>
+        <v>23982180.05</v>
       </c>
       <c r="R11">
-        <v>23816192.6450709</v>
+        <v>23816192.65</v>
       </c>
       <c r="S11">
-        <v>23650205.2373412</v>
+        <v>23650205.24</v>
       </c>
       <c r="T11">
-        <v>23484217.8296115</v>
+        <v>23484217.83</v>
       </c>
       <c r="U11">
-        <v>23262838.7264268</v>
+        <v>23262838.73</v>
       </c>
       <c r="V11">
-        <v>23041459.6232421</v>
+        <v>23041459.62</v>
       </c>
       <c r="W11">
-        <v>22820080.5200574</v>
+        <v>22820080.52</v>
       </c>
       <c r="X11">
-        <v>22598701.4168727</v>
+        <v>22598701.42</v>
       </c>
       <c r="Y11">
-        <v>22377322.313688</v>
+        <v>22377322.31</v>
       </c>
       <c r="Z11">
-        <v>22104162.687993</v>
+        <v>22104162.69</v>
       </c>
       <c r="AA11">
-        <v>21831003.062298</v>
+        <v>21831003.06</v>
       </c>
       <c r="AB11">
-        <v>21557843.436603</v>
+        <v>21557843.44</v>
       </c>
       <c r="AC11">
-        <v>21284683.810908</v>
+        <v>21284683.81</v>
       </c>
       <c r="AD11">
-        <v>21011524.185213</v>
+        <v>21011524.19</v>
       </c>
       <c r="AE11">
-        <v>20693436.1423304</v>
+        <v>20693436.14</v>
       </c>
       <c r="AF11">
-        <v>20375348.0994478</v>
+        <v>20375348.1</v>
       </c>
       <c r="AG11">
-        <v>20057260.0565652</v>
+        <v>20057260.06</v>
       </c>
       <c r="AH11">
-        <v>19739172.0136826</v>
+        <v>19739172.01</v>
       </c>
       <c r="AI11">
-        <v>19421083.9708</v>
+        <v>19421083.97</v>
       </c>
       <c r="AJ11">
-        <v>19064337.7234435</v>
+        <v>19064337.72</v>
       </c>
       <c r="AK11">
-        <v>18707591.476087</v>
+        <v>18707591.48</v>
       </c>
       <c r="AL11">
-        <v>18350845.2287305</v>
+        <v>18350845.23</v>
       </c>
       <c r="AM11">
-        <v>17994098.981374</v>
+        <v>17994098.98</v>
       </c>
       <c r="AN11">
-        <v>17637352.7340175</v>
+        <v>17637352.73</v>
       </c>
       <c r="AO11">
-        <v>17249043.5632184</v>
+        <v>17249043.56</v>
       </c>
       <c r="AP11">
-        <v>16860734.3924193</v>
+        <v>16860734.39</v>
       </c>
       <c r="AQ11">
-        <v>16472425.2216202</v>
+        <v>16472425.22</v>
       </c>
       <c r="AR11">
-        <v>16084116.0508211</v>
+        <v>16084116.05</v>
       </c>
       <c r="AS11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
       <c r="AT11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
       <c r="AU11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
       <c r="AV11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
       <c r="AW11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
       <c r="AX11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
       <c r="AY11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
       <c r="AZ11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
       <c r="BA11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
       <c r="BB11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
       <c r="BC11">
-        <v>15695806.880022</v>
+        <v>15695806.88</v>
       </c>
     </row>
     <row r="12" spans="1:55">
@@ -2283,142 +2281,142 @@
         <v>1</v>
       </c>
       <c r="J12">
-        <v>96615314.30535001</v>
+        <v>96615314.31</v>
       </c>
       <c r="K12">
-        <v>98145003.00683001</v>
+        <v>98145003.01000001</v>
       </c>
       <c r="L12">
-        <v>99655906.95642</v>
+        <v>99655906.95999999</v>
       </c>
       <c r="M12">
-        <v>101149483.21992</v>
+        <v>101149483.2</v>
       </c>
       <c r="N12">
-        <v>102626858.54876</v>
+        <v>102626858.5</v>
       </c>
       <c r="O12">
-        <v>104088700.82443</v>
+        <v>104088700.8</v>
       </c>
       <c r="P12">
-        <v>103160360.35947</v>
+        <v>103160360.4</v>
       </c>
       <c r="Q12">
-        <v>104452121.587199</v>
+        <v>104452121.6</v>
       </c>
       <c r="R12">
-        <v>105743882.814929</v>
+        <v>105743882.8</v>
       </c>
       <c r="S12">
-        <v>107035644.042659</v>
+        <v>107035644</v>
       </c>
       <c r="T12">
-        <v>108327405.270388</v>
+        <v>108327405.3</v>
       </c>
       <c r="U12">
-        <v>109535912.593573</v>
+        <v>109535912.6</v>
       </c>
       <c r="V12">
-        <v>110744419.916758</v>
+        <v>110744419.9</v>
       </c>
       <c r="W12">
-        <v>111952927.239943</v>
+        <v>111952927.2</v>
       </c>
       <c r="X12">
-        <v>113161434.563127</v>
+        <v>113161434.6</v>
       </c>
       <c r="Y12">
-        <v>114369941.886312</v>
+        <v>114369941.9</v>
       </c>
       <c r="Z12">
-        <v>115475285.912007</v>
+        <v>115475285.9</v>
       </c>
       <c r="AA12">
-        <v>116580629.937702</v>
+        <v>116580629.9</v>
       </c>
       <c r="AB12">
-        <v>117685973.963397</v>
+        <v>117685974</v>
       </c>
       <c r="AC12">
-        <v>118791317.989092</v>
+        <v>118791318</v>
       </c>
       <c r="AD12">
-        <v>119896662.014787</v>
+        <v>119896662</v>
       </c>
       <c r="AE12">
-        <v>120892736.81767</v>
+        <v>120892736.8</v>
       </c>
       <c r="AF12">
-        <v>121888811.620552</v>
+        <v>121888811.6</v>
       </c>
       <c r="AG12">
-        <v>122884886.423435</v>
+        <v>122884886.4</v>
       </c>
       <c r="AH12">
-        <v>123880961.226317</v>
+        <v>123880961.2</v>
       </c>
       <c r="AI12">
-        <v>124877036.0292</v>
+        <v>124877036</v>
       </c>
       <c r="AJ12">
-        <v>125753832.176556</v>
+        <v>125753832.2</v>
       </c>
       <c r="AK12">
-        <v>126630628.323913</v>
+        <v>126630628.3</v>
       </c>
       <c r="AL12">
-        <v>127507424.47127</v>
+        <v>127507424.5</v>
       </c>
       <c r="AM12">
-        <v>128384220.618626</v>
+        <v>128384220.6</v>
       </c>
       <c r="AN12">
-        <v>129261016.765983</v>
+        <v>129261016.8</v>
       </c>
       <c r="AO12">
-        <v>130013458.896782</v>
+        <v>130013458.9</v>
       </c>
       <c r="AP12">
-        <v>130765901.027581</v>
+        <v>130765901</v>
       </c>
       <c r="AQ12">
-        <v>131518343.15838</v>
+        <v>131518343.2</v>
       </c>
       <c r="AR12">
-        <v>132270785.289179</v>
+        <v>132270785.3</v>
       </c>
       <c r="AS12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
       <c r="AT12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
       <c r="AU12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
       <c r="AV12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
       <c r="AW12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
       <c r="AX12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
       <c r="AY12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
       <c r="AZ12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
       <c r="BA12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
       <c r="BB12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
       <c r="BC12">
-        <v>133023227.419978</v>
+        <v>133023227.4</v>
       </c>
     </row>
   </sheetData>
@@ -3082,662 +3080,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BC2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:55">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AQ1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AR1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AT1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AU1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AX1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AY1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AZ1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="BA1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="BB1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="BC1" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:55">
-      <c r="A2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-      <c r="N2">
-        <v>1</v>
-      </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
-      <c r="P2">
-        <v>1</v>
-      </c>
-      <c r="Q2">
-        <v>1</v>
-      </c>
-      <c r="R2">
-        <v>0.986842105263158</v>
-      </c>
-      <c r="S2">
-        <v>0.9736842105263158</v>
-      </c>
-      <c r="T2">
-        <v>0.9605263157894737</v>
-      </c>
-      <c r="U2">
-        <v>0.9473684210526316</v>
-      </c>
-      <c r="V2">
-        <v>0.9342105263157895</v>
-      </c>
-      <c r="W2">
-        <v>0.9210526315789473</v>
-      </c>
-      <c r="X2">
-        <v>0.9078947368421052</v>
-      </c>
-      <c r="Y2">
-        <v>0.8947368421052632</v>
-      </c>
-      <c r="Z2">
-        <v>0.8815789473684211</v>
-      </c>
-      <c r="AA2">
-        <v>0.868421052631579</v>
-      </c>
-      <c r="AB2">
-        <v>0.8552631578947368</v>
-      </c>
-      <c r="AC2">
-        <v>0.8421052631578947</v>
-      </c>
-      <c r="AD2">
-        <v>0.8289473684210527</v>
-      </c>
-      <c r="AE2">
-        <v>0.8157894736842105</v>
-      </c>
-      <c r="AF2">
-        <v>0.8026315789473684</v>
-      </c>
-      <c r="AG2">
-        <v>0.7894736842105263</v>
-      </c>
-      <c r="AH2">
-        <v>0.7763157894736842</v>
-      </c>
-      <c r="AI2">
-        <v>0.7631578947368421</v>
-      </c>
-      <c r="AJ2">
-        <v>0.75</v>
-      </c>
-      <c r="AK2">
-        <v>0.736842105263158</v>
-      </c>
-      <c r="AL2">
-        <v>0.7236842105263157</v>
-      </c>
-      <c r="AM2">
-        <v>0.7105263157894737</v>
-      </c>
-      <c r="AN2">
-        <v>0.6973684210526316</v>
-      </c>
-      <c r="AO2">
-        <v>0.6842105263157895</v>
-      </c>
-      <c r="AP2">
-        <v>0.6710526315789473</v>
-      </c>
-      <c r="AQ2">
-        <v>0.6578947368421053</v>
-      </c>
-      <c r="AR2">
-        <v>0.6447368421052632</v>
-      </c>
-      <c r="AS2">
-        <v>0.631578947368421</v>
-      </c>
-      <c r="AT2">
-        <v>0.618421052631579</v>
-      </c>
-      <c r="AU2">
-        <v>0.6052631578947368</v>
-      </c>
-      <c r="AV2">
-        <v>0.5921052631578947</v>
-      </c>
-      <c r="AW2">
-        <v>0.5789473684210527</v>
-      </c>
-      <c r="AX2">
-        <v>0.5657894736842105</v>
-      </c>
-      <c r="AY2">
-        <v>0.5526315789473684</v>
-      </c>
-      <c r="AZ2">
-        <v>0.5394736842105263</v>
-      </c>
-      <c r="BA2">
-        <v>0.5263157894736843</v>
-      </c>
-      <c r="BB2">
-        <v>0.513157894736842</v>
-      </c>
-      <c r="BC2">
-        <v>0.5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BC2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:55">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AQ1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AR1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AT1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AU1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AX1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AY1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AZ1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="BA1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="BB1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="BC1" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:55">
-      <c r="A2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-      <c r="N2">
-        <v>1</v>
-      </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
-      <c r="P2">
-        <v>1</v>
-      </c>
-      <c r="Q2">
-        <v>1</v>
-      </c>
-      <c r="R2">
-        <v>0.986842105263158</v>
-      </c>
-      <c r="S2">
-        <v>0.9736842105263158</v>
-      </c>
-      <c r="T2">
-        <v>0.9605263157894737</v>
-      </c>
-      <c r="U2">
-        <v>0.9473684210526316</v>
-      </c>
-      <c r="V2">
-        <v>0.9342105263157895</v>
-      </c>
-      <c r="W2">
-        <v>0.9210526315789473</v>
-      </c>
-      <c r="X2">
-        <v>0.9078947368421052</v>
-      </c>
-      <c r="Y2">
-        <v>0.8947368421052632</v>
-      </c>
-      <c r="Z2">
-        <v>0.8815789473684211</v>
-      </c>
-      <c r="AA2">
-        <v>0.868421052631579</v>
-      </c>
-      <c r="AB2">
-        <v>0.8552631578947368</v>
-      </c>
-      <c r="AC2">
-        <v>0.8421052631578947</v>
-      </c>
-      <c r="AD2">
-        <v>0.8289473684210527</v>
-      </c>
-      <c r="AE2">
-        <v>0.8157894736842105</v>
-      </c>
-      <c r="AF2">
-        <v>0.8026315789473684</v>
-      </c>
-      <c r="AG2">
-        <v>0.7894736842105263</v>
-      </c>
-      <c r="AH2">
-        <v>0.7763157894736842</v>
-      </c>
-      <c r="AI2">
-        <v>0.7631578947368421</v>
-      </c>
-      <c r="AJ2">
-        <v>0.75</v>
-      </c>
-      <c r="AK2">
-        <v>0.736842105263158</v>
-      </c>
-      <c r="AL2">
-        <v>0.7236842105263157</v>
-      </c>
-      <c r="AM2">
-        <v>0.7105263157894737</v>
-      </c>
-      <c r="AN2">
-        <v>0.6973684210526316</v>
-      </c>
-      <c r="AO2">
-        <v>0.6842105263157895</v>
-      </c>
-      <c r="AP2">
-        <v>0.6710526315789473</v>
-      </c>
-      <c r="AQ2">
-        <v>0.6578947368421053</v>
-      </c>
-      <c r="AR2">
-        <v>0.6447368421052632</v>
-      </c>
-      <c r="AS2">
-        <v>0.631578947368421</v>
-      </c>
-      <c r="AT2">
-        <v>0.618421052631579</v>
-      </c>
-      <c r="AU2">
-        <v>0.6052631578947368</v>
-      </c>
-      <c r="AV2">
-        <v>0.5921052631578947</v>
-      </c>
-      <c r="AW2">
-        <v>0.5789473684210527</v>
-      </c>
-      <c r="AX2">
-        <v>0.5657894736842105</v>
-      </c>
-      <c r="AY2">
-        <v>0.5526315789473684</v>
-      </c>
-      <c r="AZ2">
-        <v>0.5394736842105263</v>
-      </c>
-      <c r="BA2">
-        <v>0.5263157894736843</v>
-      </c>
-      <c r="BB2">
-        <v>0.513157894736842</v>
-      </c>
-      <c r="BC2">
-        <v>0.5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>